<commit_message>
Add aging plots and update dependency outputs
Add generated plot (PNG) and spreadsheet (XLSX) outputs for envejecimiento under output/graficos_envejecimiento (communal and regional plots across multiple regions and years 2018–2024). Also update dependency plot outputs in output/graficos_dependencia (communal PNG/XLSX and some regional XLSX files for Antofagasta, Atacama, Coquimbo, Tarapacá). These are generated assets (visualizations and data exports) produced by the analysis pipeline.
</commit_message>
<xml_diff>
--- a/output/graficos_envejecimiento/plot_comunal_d_enveje_a_2024_antofagasta.xlsx
+++ b/output/graficos_envejecimiento/plot_comunal_d_enveje_a_2024_antofagasta.xlsx
@@ -413,7 +413,7 @@
         <v>18.85489755823744</v>
       </c>
       <c r="D3">
-        <v>66.29245018243054</v>
+        <v>66.29245018243053</v>
       </c>
       <c r="E3">
         <v>14.85265225933202</v>
@@ -429,13 +429,13 @@
         <v>47.82608695652174</v>
       </c>
       <c r="C4">
-        <v>24.22752808988764</v>
+        <v>24.22752808988765</v>
       </c>
       <c r="D4">
         <v>64.18539325842697</v>
       </c>
       <c r="E4">
-        <v>11.58707865168539</v>
+        <v>11.5870786516854</v>
       </c>
     </row>
     <row r="5">
@@ -451,7 +451,7 @@
         <v>17.31067602512006</v>
       </c>
       <c r="D5">
-        <v>62.22386405615072</v>
+        <v>62.22386405615073</v>
       </c>
       <c r="E5">
         <v>20.46545991872922</v>
@@ -467,7 +467,7 @@
         <v>72.10711050724638</v>
       </c>
       <c r="C6">
-        <v>19.7653535641753</v>
+        <v>19.76535356417529</v>
       </c>
       <c r="D6">
         <v>65.98242109915687</v>
@@ -508,7 +508,7 @@
         <v>18.4655609118392</v>
       </c>
       <c r="D8">
-        <v>69.20500040853011</v>
+        <v>69.2050004085301</v>
       </c>
       <c r="E8">
         <v>12.32943867963069</v>
@@ -521,7 +521,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>105.4545454545455</v>
+        <v>105.4545454545454</v>
       </c>
       <c r="C9">
         <v>19.07443317422434</v>
@@ -540,13 +540,13 @@
         </is>
       </c>
       <c r="B10">
-        <v>90.70796460176992</v>
+        <v>90.7079646017699</v>
       </c>
       <c r="C10">
-        <v>18.15990357573322</v>
+        <v>18.15990357573323</v>
       </c>
       <c r="D10">
-        <v>65.36761751707513</v>
+        <v>65.36761751707512</v>
       </c>
       <c r="E10">
         <v>16.47247890719164</v>

</xml_diff>